<commit_message>
Fix: substituição de dados nulos
</commit_message>
<xml_diff>
--- a/base03/manteiga_metricas.xlsx
+++ b/base03/manteiga_metricas.xlsx
@@ -1046,7 +1046,9 @@
       <c r="C26" t="n">
         <v>35.23</v>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -1476,7 +1478,9 @@
       <c r="C44" t="n">
         <v>34.36</v>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -3662,7 +3666,9 @@
       <c r="C136" t="n">
         <v>35.32</v>
       </c>
-      <c r="D136" t="inlineStr"/>
+      <c r="D136" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E136" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -3948,7 +3954,9 @@
       <c r="C148" t="n">
         <v>32.22</v>
       </c>
-      <c r="D148" t="inlineStr"/>
+      <c r="D148" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E148" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -4474,7 +4482,9 @@
       <c r="C170" t="n">
         <v>32.88</v>
       </c>
-      <c r="D170" t="inlineStr"/>
+      <c r="D170" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -4520,7 +4530,9 @@
       <c r="C172" t="n">
         <v>36.35</v>
       </c>
-      <c r="D172" t="inlineStr"/>
+      <c r="D172" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
@@ -5018,7 +5030,9 @@
       <c r="C193" t="n">
         <v>31.74</v>
       </c>
-      <c r="D193" t="inlineStr"/>
+      <c r="D193" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -5280,7 +5294,9 @@
       <c r="C204" t="n">
         <v>32.52</v>
       </c>
-      <c r="D204" t="inlineStr"/>
+      <c r="D204" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E204" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -6142,7 +6158,9 @@
       <c r="C240" t="n">
         <v>32.2</v>
       </c>
-      <c r="D240" t="inlineStr"/>
+      <c r="D240" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E240" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -6712,7 +6730,9 @@
       <c r="C264" t="n">
         <v>32.46</v>
       </c>
-      <c r="D264" t="inlineStr"/>
+      <c r="D264" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E264" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -7070,7 +7090,9 @@
       <c r="C279" t="n">
         <v>36.04</v>
       </c>
-      <c r="D279" t="inlineStr"/>
+      <c r="D279" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E279" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -8048,7 +8070,9 @@
       <c r="C320" t="n">
         <v>31.62</v>
       </c>
-      <c r="D320" t="inlineStr"/>
+      <c r="D320" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E320" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -8646,7 +8670,9 @@
       <c r="C345" t="n">
         <v>33.67</v>
       </c>
-      <c r="D345" t="inlineStr"/>
+      <c r="D345" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E345" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -14692,7 +14718,9 @@
       <c r="C598" t="n">
         <v>30.27</v>
       </c>
-      <c r="D598" t="inlineStr"/>
+      <c r="D598" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E598" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -15530,7 +15558,9 @@
       <c r="C633" t="n">
         <v>32.35</v>
       </c>
-      <c r="D633" t="inlineStr"/>
+      <c r="D633" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E633" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -16704,7 +16734,9 @@
       <c r="C682" t="n">
         <v>33.14</v>
       </c>
-      <c r="D682" t="inlineStr"/>
+      <c r="D682" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E682" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -17494,7 +17526,9 @@
       <c r="C715" t="n">
         <v>28</v>
       </c>
-      <c r="D715" t="inlineStr"/>
+      <c r="D715" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E715" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -19092,7 +19126,9 @@
       <c r="C782" t="n">
         <v>33.66</v>
       </c>
-      <c r="D782" t="inlineStr"/>
+      <c r="D782" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E782" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -19786,7 +19822,9 @@
       <c r="C811" t="n">
         <v>32.68</v>
       </c>
-      <c r="D811" t="inlineStr"/>
+      <c r="D811" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E811" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -20160,7 +20198,9 @@
       <c r="C827" t="n">
         <v>37.05</v>
       </c>
-      <c r="D827" t="inlineStr"/>
+      <c r="D827" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E827" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -20638,7 +20678,9 @@
       <c r="C847" t="n">
         <v>31</v>
       </c>
-      <c r="D847" t="inlineStr"/>
+      <c r="D847" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E847" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -21500,7 +21542,9 @@
       <c r="C883" t="n">
         <v>32.53</v>
       </c>
-      <c r="D883" t="inlineStr"/>
+      <c r="D883" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E883" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -23818,7 +23862,9 @@
       <c r="C980" t="n">
         <v>33.36</v>
       </c>
-      <c r="D980" t="inlineStr"/>
+      <c r="D980" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E980" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -25228,7 +25274,9 @@
       <c r="C1039" t="n">
         <v>30.97</v>
       </c>
-      <c r="D1039" t="inlineStr"/>
+      <c r="D1039" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1039" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -27550,7 +27598,9 @@
       <c r="C1136" t="n">
         <v>33.77</v>
       </c>
-      <c r="D1136" t="inlineStr"/>
+      <c r="D1136" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1136" t="inlineStr"/>
       <c r="F1136" t="inlineStr">
         <is>
@@ -28404,7 +28454,9 @@
       <c r="C1172" t="n">
         <v>34.23</v>
       </c>
-      <c r="D1172" t="inlineStr"/>
+      <c r="D1172" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1172" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -29762,7 +29814,9 @@
       <c r="C1229" t="n">
         <v>30.83</v>
       </c>
-      <c r="D1229" t="inlineStr"/>
+      <c r="D1229" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1229" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -30840,7 +30894,9 @@
       <c r="C1274" t="n">
         <v>33.67</v>
       </c>
-      <c r="D1274" t="inlineStr"/>
+      <c r="D1274" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1274" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -32310,7 +32366,9 @@
       <c r="C1336" t="n">
         <v>31.22</v>
       </c>
-      <c r="D1336" t="inlineStr"/>
+      <c r="D1336" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1336" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -36160,7 +36218,9 @@
       <c r="C1497" t="n">
         <v>31.61</v>
       </c>
-      <c r="D1497" t="inlineStr"/>
+      <c r="D1497" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1497" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -36494,7 +36554,9 @@
       <c r="C1511" t="n">
         <v>35.28</v>
       </c>
-      <c r="D1511" t="inlineStr"/>
+      <c r="D1511" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1511" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -37516,7 +37578,9 @@
       <c r="C1554" t="n">
         <v>35.45</v>
       </c>
-      <c r="D1554" t="inlineStr"/>
+      <c r="D1554" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1554" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -38970,7 +39034,9 @@
       <c r="C1615" t="n">
         <v>36.05</v>
       </c>
-      <c r="D1615" t="inlineStr"/>
+      <c r="D1615" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1615" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -39064,7 +39130,9 @@
       <c r="C1619" t="n">
         <v>34.91</v>
       </c>
-      <c r="D1619" t="inlineStr"/>
+      <c r="D1619" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1619" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -39226,7 +39294,9 @@
       <c r="C1626" t="n">
         <v>34.74</v>
       </c>
-      <c r="D1626" t="inlineStr"/>
+      <c r="D1626" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1626" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -39488,7 +39558,9 @@
       <c r="C1637" t="n">
         <v>30.5</v>
       </c>
-      <c r="D1637" t="inlineStr"/>
+      <c r="D1637" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1637" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -39702,7 +39774,9 @@
       <c r="C1646" t="n">
         <v>33.21</v>
       </c>
-      <c r="D1646" t="inlineStr"/>
+      <c r="D1646" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1646" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -39964,7 +40038,9 @@
       <c r="C1657" t="n">
         <v>29.93</v>
       </c>
-      <c r="D1657" t="inlineStr"/>
+      <c r="D1657" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1657" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -40434,7 +40510,9 @@
       <c r="C1677" t="n">
         <v>30.97</v>
       </c>
-      <c r="D1677" t="inlineStr"/>
+      <c r="D1677" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1677" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -43836,7 +43914,9 @@
       <c r="C1819" t="n">
         <v>32.03</v>
       </c>
-      <c r="D1819" t="inlineStr"/>
+      <c r="D1819" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1819" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -44362,7 +44442,9 @@
       <c r="C1841" t="n">
         <v>33.1</v>
       </c>
-      <c r="D1841" t="inlineStr"/>
+      <c r="D1841" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1841" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -44480,7 +44562,9 @@
       <c r="C1846" t="n">
         <v>31.02</v>
       </c>
-      <c r="D1846" t="inlineStr"/>
+      <c r="D1846" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1846" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -44910,7 +44994,9 @@
       <c r="C1864" t="n">
         <v>32.36</v>
       </c>
-      <c r="D1864" t="inlineStr"/>
+      <c r="D1864" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1864" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -45124,7 +45210,9 @@
       <c r="C1873" t="n">
         <v>35.32</v>
       </c>
-      <c r="D1873" t="inlineStr"/>
+      <c r="D1873" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1873" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -47086,7 +47174,9 @@
       <c r="C1955" t="n">
         <v>32.85</v>
       </c>
-      <c r="D1955" t="inlineStr"/>
+      <c r="D1955" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E1955" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -50212,7 +50302,9 @@
       <c r="C2086" t="n">
         <v>34.14</v>
       </c>
-      <c r="D2086" t="inlineStr"/>
+      <c r="D2086" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2086" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -50686,7 +50778,9 @@
       <c r="C2106" t="n">
         <v>33.83</v>
       </c>
-      <c r="D2106" t="inlineStr"/>
+      <c r="D2106" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2106" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -51308,7 +51402,9 @@
       <c r="C2132" t="n">
         <v>34.6</v>
       </c>
-      <c r="D2132" t="inlineStr"/>
+      <c r="D2132" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2132" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -53510,7 +53606,9 @@
       <c r="C2224" t="n">
         <v>30.03</v>
       </c>
-      <c r="D2224" t="inlineStr"/>
+      <c r="D2224" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2224" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -54824,7 +54922,9 @@
       <c r="C2279" t="n">
         <v>34.67</v>
       </c>
-      <c r="D2279" t="inlineStr"/>
+      <c r="D2279" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2279" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -58070,7 +58170,9 @@
       <c r="C2415" t="n">
         <v>32.99</v>
       </c>
-      <c r="D2415" t="inlineStr"/>
+      <c r="D2415" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2415" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -58952,7 +59054,9 @@
       <c r="C2452" t="n">
         <v>33.35</v>
       </c>
-      <c r="D2452" t="inlineStr"/>
+      <c r="D2452" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2452" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -60414,7 +60518,9 @@
       <c r="C2513" t="n">
         <v>31.92</v>
       </c>
-      <c r="D2513" t="inlineStr"/>
+      <c r="D2513" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2513" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -60652,7 +60758,9 @@
       <c r="C2523" t="n">
         <v>33.03</v>
       </c>
-      <c r="D2523" t="inlineStr"/>
+      <c r="D2523" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2523" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -61106,7 +61214,9 @@
       <c r="C2542" t="n">
         <v>28</v>
       </c>
-      <c r="D2542" t="inlineStr"/>
+      <c r="D2542" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2542" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -62672,7 +62782,9 @@
       <c r="C2608" t="n">
         <v>35.33</v>
       </c>
-      <c r="D2608" t="inlineStr"/>
+      <c r="D2608" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2608" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -62886,7 +62998,9 @@
       <c r="C2617" t="n">
         <v>34.3</v>
       </c>
-      <c r="D2617" t="inlineStr"/>
+      <c r="D2617" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2617" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -62908,7 +63022,9 @@
       <c r="C2618" t="n">
         <v>33.9</v>
       </c>
-      <c r="D2618" t="inlineStr"/>
+      <c r="D2618" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2618" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -63266,7 +63382,9 @@
       <c r="C2633" t="n">
         <v>33.38</v>
       </c>
-      <c r="D2633" t="inlineStr"/>
+      <c r="D2633" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2633" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -63912,7 +64030,9 @@
       <c r="C2660" t="n">
         <v>31.84</v>
       </c>
-      <c r="D2660" t="inlineStr"/>
+      <c r="D2660" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2660" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -66710,7 +66830,9 @@
       <c r="C2777" t="n">
         <v>29.96</v>
       </c>
-      <c r="D2777" t="inlineStr"/>
+      <c r="D2777" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2777" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -66992,7 +67114,9 @@
       <c r="C2789" t="n">
         <v>34.44</v>
       </c>
-      <c r="D2789" t="inlineStr"/>
+      <c r="D2789" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2789" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -67158,7 +67282,9 @@
       <c r="C2796" t="n">
         <v>33.02</v>
       </c>
-      <c r="D2796" t="inlineStr"/>
+      <c r="D2796" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2796" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -68352,7 +68478,9 @@
       <c r="C2846" t="n">
         <v>30.24</v>
       </c>
-      <c r="D2846" t="inlineStr"/>
+      <c r="D2846" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2846" t="inlineStr"/>
       <c r="F2846" t="inlineStr">
         <is>
@@ -68490,7 +68618,9 @@
       <c r="C2852" t="n">
         <v>33.88</v>
       </c>
-      <c r="D2852" t="inlineStr"/>
+      <c r="D2852" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2852" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -68536,7 +68666,9 @@
       <c r="C2854" t="n">
         <v>34.45</v>
       </c>
-      <c r="D2854" t="inlineStr"/>
+      <c r="D2854" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2854" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -71218,7 +71350,9 @@
       <c r="C2966" t="n">
         <v>34.23</v>
       </c>
-      <c r="D2966" t="inlineStr"/>
+      <c r="D2966" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2966" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -71500,7 +71634,9 @@
       <c r="C2978" t="n">
         <v>37.22</v>
       </c>
-      <c r="D2978" t="inlineStr"/>
+      <c r="D2978" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2978" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -71570,7 +71706,9 @@
       <c r="C2981" t="n">
         <v>32.06</v>
       </c>
-      <c r="D2981" t="inlineStr"/>
+      <c r="D2981" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E2981" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -72648,7 +72786,9 @@
       <c r="C3026" t="n">
         <v>31.16</v>
       </c>
-      <c r="D3026" t="inlineStr"/>
+      <c r="D3026" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3026" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -75246,7 +75386,9 @@
       <c r="C3135" t="n">
         <v>36.21</v>
       </c>
-      <c r="D3135" t="inlineStr"/>
+      <c r="D3135" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3135" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -78664,7 +78806,9 @@
       <c r="C3278" t="n">
         <v>31.49</v>
       </c>
-      <c r="D3278" t="inlineStr"/>
+      <c r="D3278" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3278" t="inlineStr"/>
       <c r="F3278" t="inlineStr">
         <is>
@@ -79278,7 +79422,9 @@
       <c r="C3304" t="n">
         <v>33.81</v>
       </c>
-      <c r="D3304" t="inlineStr"/>
+      <c r="D3304" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3304" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -79372,7 +79518,9 @@
       <c r="C3308" t="n">
         <v>32.72</v>
       </c>
-      <c r="D3308" t="inlineStr"/>
+      <c r="D3308" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3308" t="inlineStr">
         <is>
           <t>ANVISA</t>
@@ -79442,7 +79590,9 @@
       <c r="C3311" t="n">
         <v>33.38</v>
       </c>
-      <c r="D3311" t="inlineStr"/>
+      <c r="D3311" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3311" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -80176,7 +80326,9 @@
       <c r="C3342" t="n">
         <v>33.92</v>
       </c>
-      <c r="D3342" t="inlineStr"/>
+      <c r="D3342" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3342" t="inlineStr">
         <is>
           <t>Nenhuma</t>
@@ -80438,7 +80590,9 @@
       <c r="C3353" t="n">
         <v>30.13</v>
       </c>
-      <c r="D3353" t="inlineStr"/>
+      <c r="D3353" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3353" t="inlineStr">
         <is>
           <t>Internacional</t>
@@ -80460,7 +80614,9 @@
       <c r="C3354" t="n">
         <v>36.78</v>
       </c>
-      <c r="D3354" t="inlineStr"/>
+      <c r="D3354" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3354" t="inlineStr">
         <is>
           <t>ISO-HACCP</t>
@@ -82302,7 +82458,9 @@
       <c r="C3431" t="n">
         <v>35.5</v>
       </c>
-      <c r="D3431" t="inlineStr"/>
+      <c r="D3431" t="n">
+        <v>7.826709526592636</v>
+      </c>
       <c r="E3431" t="inlineStr">
         <is>
           <t>ANVISA</t>

</xml_diff>